<commit_message>
Refresh synthetic demo data
</commit_message>
<xml_diff>
--- a/data/outputs/ev_flex_daily_trading_report_sample.xlsx
+++ b/data/outputs/ev_flex_daily_trading_report_sample.xlsx
@@ -49,7 +49,7 @@
     <t>Generated at UTC</t>
   </si>
   <si>
-    <t>2026-05-09T19:56:56.856717+00:00</t>
+    <t>2026-05-09T20:32:56.535581+00:00</t>
   </si>
   <si>
     <t>Data status</t>
@@ -595,151 +595,151 @@
     <t>suggested_action</t>
   </si>
   <si>
-    <t>2026-05-09 19:56:54.872326+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:54.901566+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:54.924245+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:54.955486+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:54.987658+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.012297+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.030211+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.055647+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.073418+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.094092+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.137166+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.162443+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.182035+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.206597+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.224074+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.242234+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.257678+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.276163+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.299966+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.324158+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.341158+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.354817+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.367830+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.385535+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.440566+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.467528+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.489635+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.520642+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.546610+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.570473+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.588130+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.613581+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.634541+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.658960+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.682695+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.708016+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.727506+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.752034+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.770381+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.788415+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.805531+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.823274+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.846934+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.870582+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.887596+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.904743+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.920455+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:55.944659+00:00</t>
-  </si>
-  <si>
-    <t>2026-05-09 19:56:56.084564+00:00</t>
+    <t>2026-05-09 20:32:54.902658+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:54.930146+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:54.952639+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:54.983582+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.010013+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.033994+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.051632+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.076897+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.094883+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.114945+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.137884+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.162872+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.182069+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.206143+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.223776+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.241574+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.257094+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.274926+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.298487+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.322554+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.339391+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.352197+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.365220+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.403804+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.453307+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.479544+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.501055+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.532169+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.558667+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.582391+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.600220+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.625581+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.643438+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.663707+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.687055+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.712072+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.731415+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.755594+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.773173+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.791205+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.807002+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.824901+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.848713+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.872504+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.889299+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.902165+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.915182+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:55.932609+00:00</t>
+  </si>
+  <si>
+    <t>2026-05-09 20:32:56.054869+00:00</t>
   </si>
   <si>
     <t>low</t>
@@ -1327,7 +1327,7 @@
     <t>MWh</t>
   </si>
   <si>
-    <t>2026-05-09T19:56:49.517408+00:00</t>
+    <t>2026-05-09T20:32:50.212572+00:00</t>
   </si>
   <si>
     <t>synthetic scenario: base</t>

</xml_diff>